<commit_message>
docs: re-verify encryption governance control
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/exchange-online-admin-checklist.xlsx
+++ b/assessment/templates/exchange-online-admin-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Exchange Online Admin" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchange Online Admin" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exchange Online Admin'!$A$4:$I$7</definedName>
@@ -598,7 +598,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Timestamped negotiated TLS handshake output for representative Microsoft 365 endpoints, including protocol, cipher suite, and certificate; Exchange connector forced-TLS or mutual-TLS configuration export where the tenant uses those mail-flow paths; Tenant-level multi-workload Customer Key DEP (`MDEP`) policy output from Get-M365DataAtRestEncryptionPolicy and tenant assignment output from Get-M365DataAtRestEncryptionPolicyAssignment, with all returned properties, plus Customer Key Onboarding Service validation or enablement state; Exchange-mailbox DEP output cannot satisfy this Copilot evidence requirement; Azure Key Vault Premium or Managed HSM evidence showing two distinct paid subscriptions, one vault or HSM per subscription for each Customer Key scenario, HSM-protected keys, 90-day recovery configuration, and purge protection; Manual Microsoft 365 service-encryption review and applicable Service Trust Portal evidence</t>
+          <t>Timestamped negotiated TLS handshake output for representative Microsoft 365 endpoints, including protocol, cipher suite, and certificate; Exchange connector forced-TLS or mutual-TLS configuration export where the tenant uses those mail-flow paths; Tenant-level multi-workload Customer Key DEP (`MDEP`) policy output from Get-M365DataAtRestEncryptionPolicy and tenant assignment output from Get-M365DataAtRestEncryptionPolicyAssignment, with all returned properties, plus Customer Key Onboarding Service validation or enablement state; Exchange-mailbox DEP output cannot satisfy this Copilot evidence requirement; Azure Key Vault or Managed HSM evidence showing two distinct paid subscriptions, one vault or HSM per subscription for each Customer Key scenario, the actual SKU, HSM-protected production keys where applicable, Azure Key Vault 90-day recovery configuration, Managed HSM recovery settings, and purge protection; Manual Microsoft 365 service-encryption review and applicable Service Trust Portal evidence</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: re-verify encryption governance control (#569)
Part of the documentation freshness program.
</commit_message>
<xml_diff>
--- a/assessment/templates/exchange-online-admin-checklist.xlsx
+++ b/assessment/templates/exchange-online-admin-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Exchange Online Admin" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchange Online Admin" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exchange Online Admin'!$A$4:$I$7</definedName>
@@ -598,7 +598,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Timestamped negotiated TLS handshake output for representative Microsoft 365 endpoints, including protocol, cipher suite, and certificate; Exchange connector forced-TLS or mutual-TLS configuration export where the tenant uses those mail-flow paths; Tenant-level multi-workload Customer Key DEP (`MDEP`) policy output from Get-M365DataAtRestEncryptionPolicy and tenant assignment output from Get-M365DataAtRestEncryptionPolicyAssignment, with all returned properties, plus Customer Key Onboarding Service validation or enablement state; Exchange-mailbox DEP output cannot satisfy this Copilot evidence requirement; Azure Key Vault Premium or Managed HSM evidence showing two distinct paid subscriptions, one vault or HSM per subscription for each Customer Key scenario, HSM-protected keys, 90-day recovery configuration, and purge protection; Manual Microsoft 365 service-encryption review and applicable Service Trust Portal evidence</t>
+          <t>Timestamped negotiated TLS handshake output for representative Microsoft 365 endpoints, including protocol, cipher suite, and certificate; Exchange connector forced-TLS or mutual-TLS configuration export where the tenant uses those mail-flow paths; Tenant-level multi-workload Customer Key DEP (`MDEP`) policy output from Get-M365DataAtRestEncryptionPolicy and tenant assignment output from Get-M365DataAtRestEncryptionPolicyAssignment, with all returned properties, plus Customer Key Onboarding Service validation or enablement state; Exchange-mailbox DEP output cannot satisfy this Copilot evidence requirement; Azure Key Vault or Managed HSM evidence showing two distinct paid subscriptions, one vault or HSM per subscription for each Customer Key scenario, the actual SKU, HSM-protected production keys where applicable, Azure Key Vault 90-day recovery configuration, Managed HSM recovery settings, and purge protection; Manual Microsoft 365 service-encryption review and applicable Service Trust Portal evidence</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>

</xml_diff>